<commit_message>
pca with different factors
</commit_message>
<xml_diff>
--- a/data/arabidopsis_datasets.xlsx
+++ b/data/arabidopsis_datasets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisabender/Studium/Bachelor thesis/Datasets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisabender/Studium/bachelor-thesis-luisa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3FEF21-031E-7C4E-B790-3D4C8229B356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724F00A3-C2C8-924A-985C-1EE621A51C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="17300" activeTab="1" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
+    <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="17300" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
   </bookViews>
   <sheets>
     <sheet name="SRA " sheetId="6" r:id="rId1"/>
@@ -4453,7 +4453,7 @@
         <v>205</v>
       </c>
       <c r="E62" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F62">
         <v>150</v>
@@ -4476,7 +4476,7 @@
         <v>205</v>
       </c>
       <c r="E63" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F63">
         <v>150</v>
@@ -4499,7 +4499,7 @@
         <v>205</v>
       </c>
       <c r="E64" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F64">
         <v>150</v>
@@ -4522,7 +4522,7 @@
         <v>205</v>
       </c>
       <c r="E65" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F65">
         <v>150</v>
@@ -4545,7 +4545,7 @@
         <v>125</v>
       </c>
       <c r="E66" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F66">
         <v>150</v>
@@ -4568,7 +4568,7 @@
         <v>205</v>
       </c>
       <c r="E67" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F67">
         <v>150</v>
@@ -4591,7 +4591,7 @@
         <v>125</v>
       </c>
       <c r="E68" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F68">
         <v>150</v>
@@ -4614,7 +4614,7 @@
         <v>125</v>
       </c>
       <c r="E69" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F69">
         <v>150</v>
@@ -4637,7 +4637,7 @@
         <v>125</v>
       </c>
       <c r="E70" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F70">
         <v>150</v>
@@ -4660,7 +4660,7 @@
         <v>125</v>
       </c>
       <c r="E71" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F71">
         <v>150</v>
@@ -4683,7 +4683,7 @@
         <v>125</v>
       </c>
       <c r="E72" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F72">
         <v>150</v>
@@ -4706,7 +4706,7 @@
         <v>205</v>
       </c>
       <c r="E73" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F73">
         <v>150</v>
@@ -4729,7 +4729,7 @@
         <v>125</v>
       </c>
       <c r="E74" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F74">
         <v>150</v>
@@ -4752,7 +4752,7 @@
         <v>125</v>
       </c>
       <c r="E75" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F75">
         <v>150</v>
@@ -4775,7 +4775,7 @@
         <v>125</v>
       </c>
       <c r="E76" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F76">
         <v>150</v>
@@ -4798,7 +4798,7 @@
         <v>205</v>
       </c>
       <c r="E77" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F77">
         <v>150</v>
@@ -4821,7 +4821,7 @@
         <v>205</v>
       </c>
       <c r="E78" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F78">
         <v>150</v>
@@ -4844,7 +4844,7 @@
         <v>205</v>
       </c>
       <c r="E79" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F79">
         <v>150</v>
@@ -12871,7 +12871,7 @@
         <v>205</v>
       </c>
       <c r="E476" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F476" s="36">
         <v>100</v>
@@ -12894,7 +12894,7 @@
         <v>205</v>
       </c>
       <c r="E477" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F477" s="36">
         <v>100</v>
@@ -12917,7 +12917,7 @@
         <v>205</v>
       </c>
       <c r="E478" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F478" s="36">
         <v>100</v>
@@ -12940,7 +12940,7 @@
         <v>205</v>
       </c>
       <c r="E479" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F479" s="36">
         <v>100</v>
@@ -12963,7 +12963,7 @@
         <v>205</v>
       </c>
       <c r="E480" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F480" s="36">
         <v>100</v>
@@ -12986,7 +12986,7 @@
         <v>205</v>
       </c>
       <c r="E481" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F481" s="36">
         <v>100</v>
@@ -13009,7 +13009,7 @@
         <v>205</v>
       </c>
       <c r="E482" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F482" s="36">
         <v>100</v>
@@ -13032,7 +13032,7 @@
         <v>205</v>
       </c>
       <c r="E483" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F483" s="36">
         <v>100</v>
@@ -13055,7 +13055,7 @@
         <v>205</v>
       </c>
       <c r="E484" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F484" s="36">
         <v>100</v>
@@ -13078,7 +13078,7 @@
         <v>731</v>
       </c>
       <c r="E485" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F485" s="36">
         <v>100</v>
@@ -13104,7 +13104,7 @@
         <v>731</v>
       </c>
       <c r="E486" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F486" s="36">
         <v>100</v>
@@ -13130,7 +13130,7 @@
         <v>731</v>
       </c>
       <c r="E487" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F487" s="36">
         <v>100</v>
@@ -13156,7 +13156,7 @@
         <v>731</v>
       </c>
       <c r="E488" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F488" s="36">
         <v>100</v>
@@ -13182,7 +13182,7 @@
         <v>731</v>
       </c>
       <c r="E489" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F489" s="36">
         <v>100</v>
@@ -13208,7 +13208,7 @@
         <v>731</v>
       </c>
       <c r="E490" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F490" s="36">
         <v>100</v>
@@ -13234,7 +13234,7 @@
         <v>731</v>
       </c>
       <c r="E491" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F491" s="36">
         <v>100</v>
@@ -13257,7 +13257,7 @@
         <v>731</v>
       </c>
       <c r="E492" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F492" s="36">
         <v>100</v>
@@ -13283,7 +13283,7 @@
         <v>731</v>
       </c>
       <c r="E493" s="36" t="s">
-        <v>206</v>
+        <v>261</v>
       </c>
       <c r="F493" s="36">
         <v>100</v>

</xml_diff>

<commit_message>
done adapter trimming on new dataset
</commit_message>
<xml_diff>
--- a/data/arabidopsis_datasets.xlsx
+++ b/data/arabidopsis_datasets.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisabender/Studium/bachelor-thesis-luisa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA06E53D-075D-DC4B-AE7A-0B03EB94E02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0F74C6-B132-6443-99A1-37014D15D6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="17180" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="1" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
   </bookViews>
   <sheets>
     <sheet name="SRA " sheetId="6" r:id="rId1"/>
     <sheet name="biotrophic" sheetId="1" r:id="rId2"/>
-    <sheet name="control" sheetId="3" r:id="rId3"/>
-    <sheet name="hemibiotrophic" sheetId="2" r:id="rId4"/>
-    <sheet name="Tabelle2" sheetId="4" r:id="rId5"/>
+    <sheet name="E.cruciferarum_new" sheetId="7" r:id="rId3"/>
+    <sheet name="control" sheetId="3" r:id="rId4"/>
+    <sheet name="hemibiotrophic" sheetId="2" r:id="rId5"/>
+    <sheet name="Tabelle2" sheetId="4" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">biotrophic!$A$1:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">E.cruciferarum_new!$A$1:$C$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SRA '!$A$1:$F$511</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3086" uniqueCount="783">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="826">
   <si>
     <t>https://www.nature.com/articles/s41598-019-56401-2</t>
   </si>
@@ -2642,6 +2644,135 @@
   </si>
   <si>
     <t>different line</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>group</t>
+  </si>
+  <si>
+    <t>sample id</t>
+  </si>
+  <si>
+    <t>1_5_S4</t>
+  </si>
+  <si>
+    <t>Col0 PM 1 dpi</t>
+  </si>
+  <si>
+    <t>1_5</t>
+  </si>
+  <si>
+    <t>1_9_S8</t>
+  </si>
+  <si>
+    <t>Col0 untr 4 dpi</t>
+  </si>
+  <si>
+    <t>1_9</t>
+  </si>
+  <si>
+    <t>2_9_S21</t>
+  </si>
+  <si>
+    <t>2_9</t>
+  </si>
+  <si>
+    <t>2_13_S25</t>
+  </si>
+  <si>
+    <t>Col0 PM 4 dpi</t>
+  </si>
+  <si>
+    <t>2_13</t>
+  </si>
+  <si>
+    <t>3_1_S29</t>
+  </si>
+  <si>
+    <t>Col0 untr 1dpi</t>
+  </si>
+  <si>
+    <t>3_9_S30</t>
+  </si>
+  <si>
+    <t>4_1_S31</t>
+  </si>
+  <si>
+    <t>4_1</t>
+  </si>
+  <si>
+    <t>4_5_S35</t>
+  </si>
+  <si>
+    <t>4_5</t>
+  </si>
+  <si>
+    <t>4_9_S39</t>
+  </si>
+  <si>
+    <t>4_9</t>
+  </si>
+  <si>
+    <t>4_13_S43</t>
+  </si>
+  <si>
+    <t>4_13</t>
+  </si>
+  <si>
+    <t>5_1_S47</t>
+  </si>
+  <si>
+    <t>5_1</t>
+  </si>
+  <si>
+    <t>5_5_S51</t>
+  </si>
+  <si>
+    <t>5_5</t>
+  </si>
+  <si>
+    <t>5_9_S55</t>
+  </si>
+  <si>
+    <t>5_9</t>
+  </si>
+  <si>
+    <t>5_13_S59</t>
+  </si>
+  <si>
+    <t>5_13</t>
+  </si>
+  <si>
+    <t>6_1_S63</t>
+  </si>
+  <si>
+    <t>6_1</t>
+  </si>
+  <si>
+    <t>6_5_S67</t>
+  </si>
+  <si>
+    <t>6_5</t>
+  </si>
+  <si>
+    <t>6_13_S74</t>
+  </si>
+  <si>
+    <t>6_13</t>
+  </si>
+  <si>
+    <t>https://hmgubox2.helmholtz-muenchen.de/index.php/s/YxREC83QWH4LXz3/download</t>
+  </si>
+  <si>
+    <t>https://hmgubox2.helmholtz-muenchen.de/index.php/s/YxREC83QWH4LXz3?path=%2FRNAseq_WT#</t>
+  </si>
+  <si>
+    <t>https://www.biorxiv.org/content/10.1101/2025.01.30.635691v1.full</t>
+  </si>
+  <si>
+    <t>Erisyphe cruciferarum (not published yet)</t>
   </si>
 </sst>
 </file>
@@ -14697,7 +14828,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FF710BC-207F-AF4F-A439-3F607FA565E9}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -15118,6 +15249,17 @@
       </c>
       <c r="G19" s="24" t="s">
         <v>185</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>825</v>
+      </c>
+      <c r="B21" t="s">
+        <v>824</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>823</v>
       </c>
     </row>
   </sheetData>
@@ -15171,6 +15313,7 @@
     <hyperlink ref="D12" r:id="rId30" display="https://www.ncbi.nlm.nih.gov/Traces/study/?acc=ERP116560&amp;o=inoculated_with_sam_s%3Ad%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%253Bacc_s%3Bacc_s%3Aa" xr:uid="{5B17F064-4B2C-094A-ADEC-C8B92FCC7C03}"/>
     <hyperlink ref="B15" r:id="rId31" location="s1" xr:uid="{9BE0D8A7-9265-8642-873F-D3EFCA103F88}"/>
     <hyperlink ref="D15" r:id="rId32" xr:uid="{10FAA8A4-AA39-A945-831D-13348C3E39A4}"/>
+    <hyperlink ref="D21" r:id="rId33" xr:uid="{FE9DC421-D5CE-8646-B5EF-C31D94D32565}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -15178,6 +15321,230 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5B0142-CAEC-C441-9ECD-DFD1FD867F69}">
+  <dimension ref="A1:D34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>783</v>
+      </c>
+      <c r="B1" t="s">
+        <v>784</v>
+      </c>
+      <c r="C1" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>786</v>
+      </c>
+      <c r="B2" t="s">
+        <v>787</v>
+      </c>
+      <c r="C2" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>789</v>
+      </c>
+      <c r="B3" t="s">
+        <v>790</v>
+      </c>
+      <c r="C3" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>792</v>
+      </c>
+      <c r="B4" t="s">
+        <v>790</v>
+      </c>
+      <c r="C4" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>794</v>
+      </c>
+      <c r="B5" t="s">
+        <v>795</v>
+      </c>
+      <c r="C5" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>797</v>
+      </c>
+      <c r="B6" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>799</v>
+      </c>
+      <c r="B7" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>800</v>
+      </c>
+      <c r="B8" t="s">
+        <v>798</v>
+      </c>
+      <c r="C8" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>802</v>
+      </c>
+      <c r="B9" t="s">
+        <v>787</v>
+      </c>
+      <c r="C9" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>804</v>
+      </c>
+      <c r="B10" t="s">
+        <v>790</v>
+      </c>
+      <c r="C10" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>806</v>
+      </c>
+      <c r="B11" t="s">
+        <v>795</v>
+      </c>
+      <c r="C11" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>808</v>
+      </c>
+      <c r="B12" t="s">
+        <v>798</v>
+      </c>
+      <c r="C12" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>810</v>
+      </c>
+      <c r="B13" t="s">
+        <v>787</v>
+      </c>
+      <c r="C13" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>812</v>
+      </c>
+      <c r="B14" t="s">
+        <v>790</v>
+      </c>
+      <c r="C14" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>814</v>
+      </c>
+      <c r="B15" t="s">
+        <v>795</v>
+      </c>
+      <c r="C15" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>816</v>
+      </c>
+      <c r="B16" t="s">
+        <v>787</v>
+      </c>
+      <c r="C16" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>818</v>
+      </c>
+      <c r="B17" t="s">
+        <v>787</v>
+      </c>
+      <c r="C17" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>820</v>
+      </c>
+      <c r="B18" t="s">
+        <v>795</v>
+      </c>
+      <c r="C18" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D32" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D33" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="34" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D34" s="19" t="s">
+        <v>823</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C18" xr:uid="{9A5B0142-CAEC-C441-9ECD-DFD1FD867F69}"/>
+  <hyperlinks>
+    <hyperlink ref="D34" r:id="rId1" xr:uid="{A1FF4488-2DC8-5146-BA94-7973ED0ED91F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F14E2C4-4692-AB49-A104-FF9B06F49CAE}">
   <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15317,7 +15684,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31891C32-2369-6E4C-B7FB-FC8E03AFC26D}">
   <dimension ref="A1:R15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15654,7 +16021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E8837A5C-3A52-8946-997E-5C0CB327FE59}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
included tissues in metadata
</commit_message>
<xml_diff>
--- a/data/arabidopsis_datasets.xlsx
+++ b/data/arabidopsis_datasets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luisabender/Studium/bachelor-thesis-luisa/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C145477-0DED-2248-8289-82A0BFC8EA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1EF4EF-C13E-4141-9CEF-3497E0779473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17260" activeTab="1" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
+    <workbookView xWindow="140" yWindow="900" windowWidth="14480" windowHeight="16860" xr2:uid="{78A52BC2-B19E-8341-BEF5-6A261385676E}"/>
   </bookViews>
   <sheets>
     <sheet name="SRA " sheetId="6" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3438" uniqueCount="835">
   <si>
     <t>https://www.nature.com/articles/s41598-019-56401-2</t>
   </si>
@@ -2565,9 +2565,6 @@
     <t>283 samples</t>
   </si>
   <si>
-    <t>bad alignment</t>
-  </si>
-  <si>
     <t>Timepoint</t>
   </si>
   <si>
@@ -2773,6 +2770,36 @@
   </si>
   <si>
     <t>Erisyphe cruciferarum (not published yet)</t>
+  </si>
+  <si>
+    <t>leaf and root</t>
+  </si>
+  <si>
+    <t>leaf</t>
+  </si>
+  <si>
+    <t>root</t>
+  </si>
+  <si>
+    <t>tissue</t>
+  </si>
+  <si>
+    <t>full aerial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leaf </t>
+  </si>
+  <si>
+    <t>whole plant</t>
+  </si>
+  <si>
+    <t>Tissue</t>
+  </si>
+  <si>
+    <t>entire seed</t>
+  </si>
+  <si>
+    <t>roots</t>
   </si>
 </sst>
 </file>
@@ -3428,7 +3455,7 @@
         <v>192</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>195</v>
@@ -3438,6 +3465,9 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>288</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>832</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -3460,7 +3490,10 @@
         <v>150</v>
       </c>
       <c r="H2" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I2" t="s">
+        <v>826</v>
       </c>
       <c r="L2" t="str">
         <f>MID(RIGHT(K2,27),1,10)</f>
@@ -3487,7 +3520,10 @@
         <v>150</v>
       </c>
       <c r="H3" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I3" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -3510,7 +3546,10 @@
         <v>150</v>
       </c>
       <c r="H4" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I4" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -3533,7 +3572,10 @@
         <v>150</v>
       </c>
       <c r="H5" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I5" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -3556,7 +3598,10 @@
         <v>150</v>
       </c>
       <c r="H6" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I6" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -3579,7 +3624,10 @@
         <v>150</v>
       </c>
       <c r="H7" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I7" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
@@ -3601,6 +3649,9 @@
       <c r="F8" s="36">
         <v>252</v>
       </c>
+      <c r="I8" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -3621,6 +3672,9 @@
       <c r="F9" s="36">
         <v>252</v>
       </c>
+      <c r="I9" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -3641,6 +3695,9 @@
       <c r="F10" s="36">
         <v>252</v>
       </c>
+      <c r="I10" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -3661,6 +3718,9 @@
       <c r="F11" s="36">
         <v>252</v>
       </c>
+      <c r="I11" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -3681,6 +3741,9 @@
       <c r="F12" s="36">
         <v>252</v>
       </c>
+      <c r="I12" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -3701,6 +3764,9 @@
       <c r="F13" s="36">
         <v>252</v>
       </c>
+      <c r="I13" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -3721,6 +3787,9 @@
       <c r="F14" s="36">
         <v>252</v>
       </c>
+      <c r="I14" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -3741,6 +3810,9 @@
       <c r="F15" s="36">
         <v>252</v>
       </c>
+      <c r="I15" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -3761,8 +3833,11 @@
       <c r="F16" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I16" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>215</v>
       </c>
@@ -3781,8 +3856,11 @@
       <c r="F17" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>216</v>
       </c>
@@ -3801,8 +3879,11 @@
       <c r="F18" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>217</v>
       </c>
@@ -3821,8 +3902,11 @@
       <c r="F19" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>218</v>
       </c>
@@ -3841,8 +3925,11 @@
       <c r="F20" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>219</v>
       </c>
@@ -3861,8 +3948,11 @@
       <c r="F21" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>220</v>
       </c>
@@ -3881,8 +3971,11 @@
       <c r="F22" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>221</v>
       </c>
@@ -3901,8 +3994,11 @@
       <c r="F23" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>222</v>
       </c>
@@ -3921,8 +4017,11 @@
       <c r="F24" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>223</v>
       </c>
@@ -3941,8 +4040,11 @@
       <c r="F25" s="36">
         <v>252</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="36" t="s">
         <v>230</v>
       </c>
@@ -3964,8 +4066,11 @@
       <c r="H26" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I26" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="36" t="s">
         <v>231</v>
       </c>
@@ -3987,8 +4092,11 @@
       <c r="H27" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I27" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="36" t="s">
         <v>232</v>
       </c>
@@ -4010,8 +4118,11 @@
       <c r="H28" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I28" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="36" t="s">
         <v>233</v>
       </c>
@@ -4033,8 +4144,11 @@
       <c r="H29" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I29" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="36" t="s">
         <v>234</v>
       </c>
@@ -4056,8 +4170,11 @@
       <c r="H30" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I30" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="36" t="s">
         <v>235</v>
       </c>
@@ -4079,8 +4196,11 @@
       <c r="H31" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I31" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="36" t="s">
         <v>236</v>
       </c>
@@ -4102,8 +4222,11 @@
       <c r="H32" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I32" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="36" t="s">
         <v>237</v>
       </c>
@@ -4125,8 +4248,11 @@
       <c r="H33" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I33" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="36" t="s">
         <v>238</v>
       </c>
@@ -4148,8 +4274,11 @@
       <c r="H34" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I34" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="36" t="s">
         <v>239</v>
       </c>
@@ -4171,8 +4300,11 @@
       <c r="H35" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I35" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="36" t="s">
         <v>240</v>
       </c>
@@ -4194,8 +4326,11 @@
       <c r="H36" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="36" t="s">
         <v>241</v>
       </c>
@@ -4217,8 +4352,11 @@
       <c r="H37" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I37" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="36" t="s">
         <v>242</v>
       </c>
@@ -4240,8 +4378,11 @@
       <c r="H38" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I38" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="36" t="s">
         <v>243</v>
       </c>
@@ -4263,8 +4404,11 @@
       <c r="H39" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I39" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="36" t="s">
         <v>244</v>
       </c>
@@ -4286,10 +4430,13 @@
       <c r="H40" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I40" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="36" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>53</v>
@@ -4309,10 +4456,13 @@
       <c r="H41" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I41" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="36" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B42" s="12" t="s">
         <v>53</v>
@@ -4332,10 +4482,13 @@
       <c r="H42" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I42" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="36" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B43" s="12" t="s">
         <v>53</v>
@@ -4355,10 +4508,13 @@
       <c r="H43" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I43" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="36" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="B44" s="12" t="s">
         <v>53</v>
@@ -4378,10 +4534,13 @@
       <c r="H44" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I44" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="36" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B45" s="12" t="s">
         <v>53</v>
@@ -4401,10 +4560,13 @@
       <c r="H45" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I45" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="36" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B46" s="12" t="s">
         <v>53</v>
@@ -4424,10 +4586,13 @@
       <c r="H46" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I46" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="36" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>53</v>
@@ -4447,10 +4612,13 @@
       <c r="H47" s="36" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I47" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="36" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>53</v>
@@ -4470,10 +4638,13 @@
       <c r="H48" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I48" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="36" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>53</v>
@@ -4493,10 +4664,13 @@
       <c r="H49" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I49" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="36" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B50" s="12" t="s">
         <v>53</v>
@@ -4516,10 +4690,13 @@
       <c r="H50" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I50" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="36" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="B51" s="12" t="s">
         <v>53</v>
@@ -4539,10 +4716,13 @@
       <c r="H51" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I51" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="36" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B52" s="12" t="s">
         <v>53</v>
@@ -4562,10 +4742,13 @@
       <c r="H52" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I52" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="36" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B53" s="12" t="s">
         <v>53</v>
@@ -4585,10 +4768,13 @@
       <c r="H53" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I53" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="36" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B54" s="12" t="s">
         <v>53</v>
@@ -4608,10 +4794,13 @@
       <c r="H54" s="36" t="s">
         <v>287</v>
       </c>
+      <c r="I54" t="s">
+        <v>826</v>
+      </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="36" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B55" s="12" t="s">
         <v>53</v>
@@ -4630,6 +4819,9 @@
       </c>
       <c r="H55" s="36" t="s">
         <v>287</v>
+      </c>
+      <c r="I55" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
@@ -4655,7 +4847,7 @@
         <v>287</v>
       </c>
       <c r="J56" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
@@ -4681,7 +4873,7 @@
         <v>287</v>
       </c>
       <c r="J57" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
@@ -4707,7 +4899,7 @@
         <v>287</v>
       </c>
       <c r="J58" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
@@ -4733,7 +4925,7 @@
         <v>287</v>
       </c>
       <c r="J59" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
@@ -4759,7 +4951,7 @@
         <v>287</v>
       </c>
       <c r="J60" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
@@ -4785,7 +4977,7 @@
         <v>287</v>
       </c>
       <c r="J61" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
@@ -4811,7 +5003,7 @@
         <v>287</v>
       </c>
       <c r="J62" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
@@ -4837,7 +5029,7 @@
         <v>287</v>
       </c>
       <c r="J63" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
@@ -4863,7 +5055,7 @@
         <v>287</v>
       </c>
       <c r="J64" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.2">
@@ -4889,7 +5081,7 @@
         <v>287</v>
       </c>
       <c r="J65" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
@@ -4915,7 +5107,7 @@
         <v>287</v>
       </c>
       <c r="J66" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.2">
@@ -4941,7 +5133,7 @@
         <v>287</v>
       </c>
       <c r="J67" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
@@ -4967,7 +5159,7 @@
         <v>287</v>
       </c>
       <c r="J68" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.2">
@@ -4993,7 +5185,7 @@
         <v>287</v>
       </c>
       <c r="J69" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.2">
@@ -5019,7 +5211,7 @@
         <v>287</v>
       </c>
       <c r="J70" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
@@ -5161,6 +5353,9 @@
       <c r="F77">
         <v>150</v>
       </c>
+      <c r="I77" t="s">
+        <v>827</v>
+      </c>
       <c r="L77" t="s">
         <v>748</v>
       </c>
@@ -5184,6 +5379,9 @@
       <c r="F78">
         <v>150</v>
       </c>
+      <c r="I78" t="s">
+        <v>827</v>
+      </c>
       <c r="L78" t="s">
         <v>748</v>
       </c>
@@ -5207,6 +5405,9 @@
       <c r="F79">
         <v>150</v>
       </c>
+      <c r="I79" t="s">
+        <v>827</v>
+      </c>
       <c r="L79" t="s">
         <v>748</v>
       </c>
@@ -5230,6 +5431,9 @@
       <c r="F80">
         <v>150</v>
       </c>
+      <c r="I80" t="s">
+        <v>827</v>
+      </c>
       <c r="L80" t="s">
         <v>748</v>
       </c>
@@ -5253,6 +5457,9 @@
       <c r="F81">
         <v>150</v>
       </c>
+      <c r="I81" t="s">
+        <v>827</v>
+      </c>
       <c r="L81" t="s">
         <v>748</v>
       </c>
@@ -5276,6 +5483,9 @@
       <c r="F82">
         <v>150</v>
       </c>
+      <c r="I82" t="s">
+        <v>827</v>
+      </c>
       <c r="L82" t="s">
         <v>748</v>
       </c>
@@ -5299,6 +5509,9 @@
       <c r="F83">
         <v>150</v>
       </c>
+      <c r="I83" t="s">
+        <v>827</v>
+      </c>
       <c r="L83" t="s">
         <v>748</v>
       </c>
@@ -5322,6 +5535,9 @@
       <c r="F84">
         <v>150</v>
       </c>
+      <c r="I84" t="s">
+        <v>827</v>
+      </c>
       <c r="L84" t="s">
         <v>748</v>
       </c>
@@ -5345,6 +5561,9 @@
       <c r="F85">
         <v>150</v>
       </c>
+      <c r="I85" t="s">
+        <v>827</v>
+      </c>
       <c r="L85" t="s">
         <v>748</v>
       </c>
@@ -5368,6 +5587,9 @@
       <c r="F86">
         <v>150</v>
       </c>
+      <c r="I86" t="s">
+        <v>827</v>
+      </c>
       <c r="L86" t="s">
         <v>748</v>
       </c>
@@ -5391,6 +5613,9 @@
       <c r="F87">
         <v>150</v>
       </c>
+      <c r="I87" t="s">
+        <v>827</v>
+      </c>
       <c r="L87" t="s">
         <v>748</v>
       </c>
@@ -5414,6 +5639,9 @@
       <c r="F88">
         <v>150</v>
       </c>
+      <c r="I88" t="s">
+        <v>827</v>
+      </c>
       <c r="L88" t="s">
         <v>748</v>
       </c>
@@ -5437,6 +5665,9 @@
       <c r="F89">
         <v>150</v>
       </c>
+      <c r="I89" t="s">
+        <v>827</v>
+      </c>
       <c r="L89" t="s">
         <v>748</v>
       </c>
@@ -5460,6 +5691,9 @@
       <c r="F90">
         <v>150</v>
       </c>
+      <c r="I90" t="s">
+        <v>827</v>
+      </c>
       <c r="L90" t="s">
         <v>748</v>
       </c>
@@ -5483,6 +5717,9 @@
       <c r="F91">
         <v>150</v>
       </c>
+      <c r="I91" t="s">
+        <v>827</v>
+      </c>
       <c r="L91" t="s">
         <v>748</v>
       </c>
@@ -5506,6 +5743,9 @@
       <c r="F92">
         <v>150</v>
       </c>
+      <c r="I92" t="s">
+        <v>827</v>
+      </c>
       <c r="L92" t="s">
         <v>748</v>
       </c>
@@ -5529,6 +5769,9 @@
       <c r="F93">
         <v>150</v>
       </c>
+      <c r="I93" t="s">
+        <v>827</v>
+      </c>
       <c r="L93" t="s">
         <v>748</v>
       </c>
@@ -5552,6 +5795,9 @@
       <c r="F94">
         <v>150</v>
       </c>
+      <c r="I94" t="s">
+        <v>827</v>
+      </c>
       <c r="L94" t="s">
         <v>748</v>
       </c>
@@ -9498,6 +9744,9 @@
       <c r="H291" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I291" s="36" t="s">
+        <v>831</v>
+      </c>
       <c r="J291" t="s">
         <v>750</v>
       </c>
@@ -9524,6 +9773,9 @@
       <c r="H292" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I292" s="36" t="s">
+        <v>831</v>
+      </c>
       <c r="J292" t="s">
         <v>751</v>
       </c>
@@ -9550,6 +9802,9 @@
       <c r="H293" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I293" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="294" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A294" s="50" t="s">
@@ -9573,6 +9828,9 @@
       <c r="H294" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I294" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="295" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A295" s="50" t="s">
@@ -9596,6 +9854,9 @@
       <c r="H295" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I295" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="296" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A296" s="50" t="s">
@@ -9619,6 +9880,9 @@
       <c r="H296" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I296" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="297" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A297" s="50" t="s">
@@ -9642,6 +9906,9 @@
       <c r="H297" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I297" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="298" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A298" s="50" t="s">
@@ -9665,6 +9932,9 @@
       <c r="H298" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I298" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="299" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A299" s="50" t="s">
@@ -9688,6 +9958,9 @@
       <c r="H299" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I299" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="300" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A300" s="50" t="s">
@@ -9711,6 +9984,9 @@
       <c r="H300" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I300" s="36" t="s">
+        <v>831</v>
+      </c>
       <c r="M300">
         <v>85</v>
       </c>
@@ -9737,6 +10013,9 @@
       <c r="H301" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I301" s="36" t="s">
+        <v>831</v>
+      </c>
       <c r="M301">
         <v>100</v>
       </c>
@@ -9763,6 +10042,9 @@
       <c r="H302" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I302" s="36" t="s">
+        <v>831</v>
+      </c>
       <c r="M302">
         <v>150</v>
       </c>
@@ -9789,6 +10071,9 @@
       <c r="H303" s="36" t="s">
         <v>749</v>
       </c>
+      <c r="I303" s="36" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="304" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A304" s="50" t="s">
@@ -9812,8 +10097,11 @@
       <c r="H304" s="36" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="305" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I304" s="36" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="305" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A305" s="50" t="s">
         <v>505</v>
       </c>
@@ -9835,8 +10123,11 @@
       <c r="H305" s="36" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="306" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I305" s="36" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="306" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A306" s="50" t="s">
         <v>506</v>
       </c>
@@ -9858,8 +10149,11 @@
       <c r="H306" s="36" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="307" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I306" s="36" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="307" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A307" s="50" t="s">
         <v>507</v>
       </c>
@@ -9881,8 +10175,11 @@
       <c r="H307" s="36" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="308" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I307" s="36" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A308" s="50" t="s">
         <v>508</v>
       </c>
@@ -9904,8 +10201,11 @@
       <c r="H308" s="36" t="s">
         <v>749</v>
       </c>
-    </row>
-    <row r="309" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I308" s="36" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A309" s="36" t="s">
         <v>510</v>
       </c>
@@ -9927,8 +10227,11 @@
       <c r="H309" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="310" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I309" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A310" s="36" t="s">
         <v>511</v>
       </c>
@@ -9950,8 +10253,11 @@
       <c r="H310" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="311" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I310" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A311" s="36" t="s">
         <v>512</v>
       </c>
@@ -9973,8 +10279,11 @@
       <c r="H311" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="312" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I311" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A312" s="36" t="s">
         <v>513</v>
       </c>
@@ -9996,8 +10305,11 @@
       <c r="H312" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="313" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I312" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A313" s="36" t="s">
         <v>514</v>
       </c>
@@ -10019,8 +10331,11 @@
       <c r="H313" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="314" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I313" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A314" s="36" t="s">
         <v>515</v>
       </c>
@@ -10042,8 +10357,11 @@
       <c r="H314" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="315" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I314" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="315" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A315" s="36" t="s">
         <v>516</v>
       </c>
@@ -10065,8 +10383,11 @@
       <c r="H315" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="316" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I315" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="316" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A316" s="36" t="s">
         <v>517</v>
       </c>
@@ -10088,8 +10409,11 @@
       <c r="H316" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="317" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I316" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="317" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A317" s="36" t="s">
         <v>518</v>
       </c>
@@ -10111,8 +10435,11 @@
       <c r="H317" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="318" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I317" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="318" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A318" s="36" t="s">
         <v>519</v>
       </c>
@@ -10134,8 +10461,11 @@
       <c r="H318" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="319" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I318" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="319" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A319" s="36" t="s">
         <v>520</v>
       </c>
@@ -10157,8 +10487,11 @@
       <c r="H319" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="320" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I319" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="320" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A320" s="36" t="s">
         <v>521</v>
       </c>
@@ -10180,8 +10513,11 @@
       <c r="H320" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="321" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I320" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A321" s="36" t="s">
         <v>522</v>
       </c>
@@ -10203,8 +10539,11 @@
       <c r="H321" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="322" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I321" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A322" s="36" t="s">
         <v>523</v>
       </c>
@@ -10226,8 +10565,11 @@
       <c r="H322" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="323" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I322" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A323" s="36" t="s">
         <v>524</v>
       </c>
@@ -10249,8 +10591,11 @@
       <c r="H323" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="324" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I323" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A324" s="36" t="s">
         <v>525</v>
       </c>
@@ -10272,8 +10617,11 @@
       <c r="H324" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="325" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I324" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A325" s="36" t="s">
         <v>526</v>
       </c>
@@ -10295,8 +10643,11 @@
       <c r="H325" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="326" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I325" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A326" s="36" t="s">
         <v>527</v>
       </c>
@@ -10318,8 +10669,11 @@
       <c r="H326" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="327" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I326" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A327" s="36" t="s">
         <v>528</v>
       </c>
@@ -10341,8 +10695,11 @@
       <c r="H327" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I327" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A328" s="36" t="s">
         <v>529</v>
       </c>
@@ -10364,8 +10721,11 @@
       <c r="H328" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I328" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A329" s="36" t="s">
         <v>530</v>
       </c>
@@ -10387,8 +10747,11 @@
       <c r="H329" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I329" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="330" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A330" s="36" t="s">
         <v>531</v>
       </c>
@@ -10410,8 +10773,11 @@
       <c r="H330" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I330" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="331" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A331" s="36" t="s">
         <v>532</v>
       </c>
@@ -10433,8 +10799,11 @@
       <c r="H331" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I331" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="332" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A332" s="36" t="s">
         <v>533</v>
       </c>
@@ -10456,8 +10825,11 @@
       <c r="H332" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I332" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="333" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A333" s="36" t="s">
         <v>534</v>
       </c>
@@ -10479,8 +10851,11 @@
       <c r="H333" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="334" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I333" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="334" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A334" s="36" t="s">
         <v>535</v>
       </c>
@@ -10502,8 +10877,11 @@
       <c r="H334" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I334" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="335" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A335" s="36" t="s">
         <v>536</v>
       </c>
@@ -10525,8 +10903,11 @@
       <c r="H335" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I335" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="336" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A336" s="36" t="s">
         <v>537</v>
       </c>
@@ -10548,8 +10929,11 @@
       <c r="H336" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I336" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="337" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A337" s="36" t="s">
         <v>538</v>
       </c>
@@ -10571,8 +10955,11 @@
       <c r="H337" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I337" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="338" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A338" s="36" t="s">
         <v>539</v>
       </c>
@@ -10594,8 +10981,11 @@
       <c r="H338" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="339" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I338" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="339" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A339" s="36" t="s">
         <v>540</v>
       </c>
@@ -10617,8 +11007,11 @@
       <c r="H339" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="340" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I339" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="340" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A340" s="36" t="s">
         <v>541</v>
       </c>
@@ -10640,8 +11033,11 @@
       <c r="H340" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I340" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A341" s="36" t="s">
         <v>542</v>
       </c>
@@ -10663,8 +11059,11 @@
       <c r="H341" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="342" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I341" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="342" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A342" s="36" t="s">
         <v>543</v>
       </c>
@@ -10686,8 +11085,11 @@
       <c r="H342" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="343" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I342" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A343" s="36" t="s">
         <v>544</v>
       </c>
@@ -10709,8 +11111,11 @@
       <c r="H343" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="344" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I343" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="344" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A344" s="36" t="s">
         <v>545</v>
       </c>
@@ -10732,8 +11137,11 @@
       <c r="H344" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="345" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I344" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="345" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A345" s="36" t="s">
         <v>546</v>
       </c>
@@ -10755,8 +11163,11 @@
       <c r="H345" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="346" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I345" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="346" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A346" s="36" t="s">
         <v>547</v>
       </c>
@@ -10778,8 +11189,11 @@
       <c r="H346" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="347" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I346" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="347" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A347" s="36" t="s">
         <v>548</v>
       </c>
@@ -10801,8 +11215,11 @@
       <c r="H347" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="348" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I347" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="348" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A348" s="36" t="s">
         <v>549</v>
       </c>
@@ -10824,8 +11241,11 @@
       <c r="H348" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="349" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I348" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="349" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A349" s="36" t="s">
         <v>550</v>
       </c>
@@ -10847,8 +11267,11 @@
       <c r="H349" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="350" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I349" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="350" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A350" s="36" t="s">
         <v>551</v>
       </c>
@@ -10870,8 +11293,11 @@
       <c r="H350" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="351" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I350" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="351" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A351" s="36" t="s">
         <v>552</v>
       </c>
@@ -10893,8 +11319,11 @@
       <c r="H351" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="352" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I351" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="352" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A352" s="36" t="s">
         <v>553</v>
       </c>
@@ -10916,8 +11345,11 @@
       <c r="H352" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="353" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I352" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="353" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A353" s="36" t="s">
         <v>554</v>
       </c>
@@ -10939,8 +11371,11 @@
       <c r="H353" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="354" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I353" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="354" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A354" s="36" t="s">
         <v>555</v>
       </c>
@@ -10962,8 +11397,11 @@
       <c r="H354" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="355" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I354" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="355" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A355" s="36" t="s">
         <v>556</v>
       </c>
@@ -10985,8 +11423,11 @@
       <c r="H355" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="356" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I355" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="356" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A356" s="36" t="s">
         <v>557</v>
       </c>
@@ -11008,8 +11449,11 @@
       <c r="H356" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="357" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I356" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="357" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A357" s="36" t="s">
         <v>558</v>
       </c>
@@ -11031,8 +11475,11 @@
       <c r="H357" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="358" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I357" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A358" s="36" t="s">
         <v>559</v>
       </c>
@@ -11054,8 +11501,11 @@
       <c r="H358" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="359" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I358" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A359" s="36" t="s">
         <v>560</v>
       </c>
@@ -11077,8 +11527,11 @@
       <c r="H359" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="360" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I359" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A360" s="36" t="s">
         <v>561</v>
       </c>
@@ -11100,8 +11553,11 @@
       <c r="H360" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="361" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I360" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A361" s="36" t="s">
         <v>562</v>
       </c>
@@ -11123,8 +11579,11 @@
       <c r="H361" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="362" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I361" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A362" s="36" t="s">
         <v>563</v>
       </c>
@@ -11146,8 +11605,11 @@
       <c r="H362" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="363" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I362" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A363" s="36" t="s">
         <v>564</v>
       </c>
@@ -11169,8 +11631,11 @@
       <c r="H363" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I363" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A364" s="36" t="s">
         <v>565</v>
       </c>
@@ -11192,8 +11657,11 @@
       <c r="H364" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="365" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I364" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A365" s="36" t="s">
         <v>566</v>
       </c>
@@ -11215,8 +11683,11 @@
       <c r="H365" s="36" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="366" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I365" s="36" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="366" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A366" s="36" t="s">
         <v>569</v>
       </c>
@@ -11235,8 +11706,11 @@
       <c r="F366" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="367" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I366" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="367" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A367" s="36" t="s">
         <v>570</v>
       </c>
@@ -11255,8 +11729,11 @@
       <c r="F367" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="368" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I367" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A368" s="36" t="s">
         <v>571</v>
       </c>
@@ -11275,8 +11752,11 @@
       <c r="F368" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="369" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I368" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="369" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A369" s="36" t="s">
         <v>572</v>
       </c>
@@ -11295,8 +11775,11 @@
       <c r="F369" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="370" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I369" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="370" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A370" s="36" t="s">
         <v>573</v>
       </c>
@@ -11315,8 +11798,11 @@
       <c r="F370" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="371" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I370" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="371" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A371" s="36" t="s">
         <v>574</v>
       </c>
@@ -11335,8 +11821,11 @@
       <c r="F371" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="372" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I371" s="36" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="372" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A372" s="36" t="s">
         <v>575</v>
       </c>
@@ -11355,8 +11844,11 @@
       <c r="F372" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="373" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I372" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="373" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A373" s="36" t="s">
         <v>576</v>
       </c>
@@ -11375,8 +11867,11 @@
       <c r="F373" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="374" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I373" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="374" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A374" s="36" t="s">
         <v>577</v>
       </c>
@@ -11395,8 +11890,11 @@
       <c r="F374" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="375" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I374" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="375" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A375" s="36" t="s">
         <v>578</v>
       </c>
@@ -11415,8 +11913,11 @@
       <c r="F375" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="376" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I375" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="376" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A376" s="36" t="s">
         <v>579</v>
       </c>
@@ -11435,8 +11936,11 @@
       <c r="F376" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="377" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I376" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="377" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A377" s="36" t="s">
         <v>580</v>
       </c>
@@ -11455,8 +11959,11 @@
       <c r="F377" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="378" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I377" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="378" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A378" s="36" t="s">
         <v>581</v>
       </c>
@@ -11475,8 +11982,11 @@
       <c r="F378" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="379" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I378" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="379" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A379" s="36" t="s">
         <v>582</v>
       </c>
@@ -11495,8 +12005,11 @@
       <c r="F379" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="380" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I379" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="380" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A380" s="36" t="s">
         <v>583</v>
       </c>
@@ -11515,8 +12028,11 @@
       <c r="F380" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="381" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I380" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="381" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A381" s="36" t="s">
         <v>587</v>
       </c>
@@ -11535,8 +12051,11 @@
       <c r="F381" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="382" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I381" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="382" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A382" s="36" t="s">
         <v>588</v>
       </c>
@@ -11555,8 +12074,11 @@
       <c r="F382" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="383" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I382" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="383" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A383" s="36" t="s">
         <v>589</v>
       </c>
@@ -11575,8 +12097,11 @@
       <c r="F383" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="384" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I383" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="384" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A384" s="36" t="s">
         <v>590</v>
       </c>
@@ -11595,8 +12120,11 @@
       <c r="F384" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="385" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I384" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="385" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A385" s="36" t="s">
         <v>591</v>
       </c>
@@ -11615,8 +12143,11 @@
       <c r="F385" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="386" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I385" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="386" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A386" s="36" t="s">
         <v>592</v>
       </c>
@@ -11635,8 +12166,11 @@
       <c r="F386" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="387" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I386" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="387" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A387" s="36" t="s">
         <v>593</v>
       </c>
@@ -11655,8 +12189,11 @@
       <c r="F387" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="388" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I387" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="388" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A388" s="36" t="s">
         <v>594</v>
       </c>
@@ -11675,8 +12212,11 @@
       <c r="F388" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="389" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I388" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="389" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A389" s="36" t="s">
         <v>595</v>
       </c>
@@ -11695,8 +12235,11 @@
       <c r="F389" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I389" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="390" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A390" s="36" t="s">
         <v>596</v>
       </c>
@@ -11715,8 +12258,11 @@
       <c r="F390" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="391" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I390" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="391" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A391" s="36" t="s">
         <v>597</v>
       </c>
@@ -11735,8 +12281,11 @@
       <c r="F391" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="392" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I391" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="392" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A392" s="36" t="s">
         <v>598</v>
       </c>
@@ -11755,8 +12304,11 @@
       <c r="F392" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="393" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I392" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="393" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A393" s="36" t="s">
         <v>599</v>
       </c>
@@ -11775,8 +12327,11 @@
       <c r="F393" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="394" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I393" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="394" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A394" s="36" t="s">
         <v>600</v>
       </c>
@@ -11795,8 +12350,11 @@
       <c r="F394" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="395" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I394" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="395" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A395" s="36" t="s">
         <v>601</v>
       </c>
@@ -11815,8 +12373,11 @@
       <c r="F395" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="396" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I395" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="396" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A396" s="36" t="s">
         <v>602</v>
       </c>
@@ -11835,8 +12396,11 @@
       <c r="F396" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="397" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I396" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="397" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A397" s="36" t="s">
         <v>603</v>
       </c>
@@ -11855,8 +12419,11 @@
       <c r="F397" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="398" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I397" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="398" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A398" s="36" t="s">
         <v>604</v>
       </c>
@@ -11875,8 +12442,11 @@
       <c r="F398" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="399" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I398" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="399" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A399" s="36" t="s">
         <v>605</v>
       </c>
@@ -11895,8 +12465,11 @@
       <c r="F399" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="400" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I399" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="400" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A400" s="36" t="s">
         <v>606</v>
       </c>
@@ -11915,8 +12488,11 @@
       <c r="F400" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="401" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I400" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="401" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A401" s="36" t="s">
         <v>607</v>
       </c>
@@ -11935,8 +12511,11 @@
       <c r="F401" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="402" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I401" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="402" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A402" s="36" t="s">
         <v>608</v>
       </c>
@@ -11955,8 +12534,11 @@
       <c r="F402" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="403" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I402" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="403" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A403" s="36" t="s">
         <v>609</v>
       </c>
@@ -11975,8 +12557,11 @@
       <c r="F403" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="404" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I403" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="404" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A404" s="36" t="s">
         <v>610</v>
       </c>
@@ -11995,8 +12580,11 @@
       <c r="F404" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="405" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I404" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="405" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A405" s="36" t="s">
         <v>611</v>
       </c>
@@ -12015,8 +12603,11 @@
       <c r="F405" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="406" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I405" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="406" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A406" s="36" t="s">
         <v>612</v>
       </c>
@@ -12035,8 +12626,11 @@
       <c r="F406" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="407" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I406" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="407" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A407" s="36" t="s">
         <v>613</v>
       </c>
@@ -12055,8 +12649,11 @@
       <c r="F407" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="408" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I407" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="408" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A408" s="36" t="s">
         <v>614</v>
       </c>
@@ -12075,8 +12672,11 @@
       <c r="F408" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="409" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I408" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="409" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A409" s="36" t="s">
         <v>615</v>
       </c>
@@ -12095,8 +12695,11 @@
       <c r="F409" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="410" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I409" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="410" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A410" s="36" t="s">
         <v>616</v>
       </c>
@@ -12115,8 +12718,11 @@
       <c r="F410" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="411" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I410" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="411" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A411" s="36" t="s">
         <v>617</v>
       </c>
@@ -12135,8 +12741,11 @@
       <c r="F411" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="412" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I411" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="412" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A412" s="36" t="s">
         <v>618</v>
       </c>
@@ -12155,8 +12764,11 @@
       <c r="F412" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I412" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="413" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A413" s="36" t="s">
         <v>619</v>
       </c>
@@ -12175,8 +12787,11 @@
       <c r="F413" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="414" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I413" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="414" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A414" s="36" t="s">
         <v>620</v>
       </c>
@@ -12195,8 +12810,11 @@
       <c r="F414" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="415" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I414" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="415" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A415" s="36" t="s">
         <v>621</v>
       </c>
@@ -12215,8 +12833,11 @@
       <c r="F415" s="36">
         <v>202</v>
       </c>
-    </row>
-    <row r="416" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I415" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="416" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A416" s="36" t="s">
         <v>622</v>
       </c>
@@ -12234,6 +12855,9 @@
       </c>
       <c r="F416" s="36">
         <v>202</v>
+      </c>
+      <c r="I416" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="417" spans="1:10" x14ac:dyDescent="0.2">
@@ -12244,7 +12868,7 @@
         <v>121</v>
       </c>
       <c r="C417" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D417" s="36" t="s">
         <v>654</v>
@@ -12258,8 +12882,11 @@
       <c r="H417" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I417" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J417" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="418" spans="1:10" x14ac:dyDescent="0.2">
@@ -12270,7 +12897,7 @@
         <v>121</v>
       </c>
       <c r="C418" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D418" s="36" t="s">
         <v>204</v>
@@ -12284,8 +12911,11 @@
       <c r="H418" s="36" t="s">
         <v>657</v>
       </c>
+      <c r="I418" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J418" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="419" spans="1:10" x14ac:dyDescent="0.2">
@@ -12296,7 +12926,7 @@
         <v>121</v>
       </c>
       <c r="C419" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D419" s="36" t="s">
         <v>204</v>
@@ -12309,6 +12939,9 @@
       </c>
       <c r="H419" s="36" t="s">
         <v>657</v>
+      </c>
+      <c r="I419" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="420" spans="1:10" x14ac:dyDescent="0.2">
@@ -12319,7 +12952,7 @@
         <v>121</v>
       </c>
       <c r="C420" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D420" s="36" t="s">
         <v>204</v>
@@ -12332,6 +12965,9 @@
       </c>
       <c r="H420" s="36" t="s">
         <v>657</v>
+      </c>
+      <c r="I420" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="421" spans="1:10" x14ac:dyDescent="0.2">
@@ -12342,7 +12978,7 @@
         <v>121</v>
       </c>
       <c r="C421" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D421" s="36" t="s">
         <v>204</v>
@@ -12355,6 +12991,9 @@
       </c>
       <c r="H421" s="36" t="s">
         <v>658</v>
+      </c>
+      <c r="I421" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="422" spans="1:10" x14ac:dyDescent="0.2">
@@ -12365,7 +13004,7 @@
         <v>121</v>
       </c>
       <c r="C422" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D422" s="36" t="s">
         <v>204</v>
@@ -12378,6 +13017,9 @@
       </c>
       <c r="H422" s="36" t="s">
         <v>658</v>
+      </c>
+      <c r="I422" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="423" spans="1:10" x14ac:dyDescent="0.2">
@@ -12388,7 +13030,7 @@
         <v>121</v>
       </c>
       <c r="C423" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D423" s="36" t="s">
         <v>204</v>
@@ -12401,6 +13043,9 @@
       </c>
       <c r="H423" s="36" t="s">
         <v>658</v>
+      </c>
+      <c r="I423" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="424" spans="1:10" x14ac:dyDescent="0.2">
@@ -12411,7 +13056,7 @@
         <v>121</v>
       </c>
       <c r="C424" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D424" s="36" t="s">
         <v>655</v>
@@ -12425,8 +13070,11 @@
       <c r="H424" s="36" t="s">
         <v>657</v>
       </c>
+      <c r="I424" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J424" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="425" spans="1:10" x14ac:dyDescent="0.2">
@@ -12437,7 +13085,7 @@
         <v>121</v>
       </c>
       <c r="C425" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D425" s="36" t="s">
         <v>655</v>
@@ -12451,11 +13099,11 @@
       <c r="H425" s="36" t="s">
         <v>657</v>
       </c>
-      <c r="I425" t="s">
-        <v>756</v>
+      <c r="I425" s="36" t="s">
+        <v>829</v>
       </c>
       <c r="J425" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="426" spans="1:10" x14ac:dyDescent="0.2">
@@ -12466,7 +13114,7 @@
         <v>121</v>
       </c>
       <c r="C426" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D426" s="36" t="s">
         <v>655</v>
@@ -12480,11 +13128,11 @@
       <c r="H426" s="36" t="s">
         <v>657</v>
       </c>
-      <c r="I426" t="s">
-        <v>756</v>
+      <c r="I426" s="36" t="s">
+        <v>829</v>
       </c>
       <c r="J426" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="427" spans="1:10" x14ac:dyDescent="0.2">
@@ -12495,7 +13143,7 @@
         <v>121</v>
       </c>
       <c r="C427" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D427" s="36" t="s">
         <v>655</v>
@@ -12509,8 +13157,11 @@
       <c r="H427" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I427" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J427" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="428" spans="1:10" x14ac:dyDescent="0.2">
@@ -12521,7 +13172,7 @@
         <v>121</v>
       </c>
       <c r="C428" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D428" s="36" t="s">
         <v>655</v>
@@ -12535,8 +13186,11 @@
       <c r="H428" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I428" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J428" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="429" spans="1:10" x14ac:dyDescent="0.2">
@@ -12547,7 +13201,7 @@
         <v>121</v>
       </c>
       <c r="C429" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D429" s="36" t="s">
         <v>655</v>
@@ -12561,8 +13215,11 @@
       <c r="H429" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I429" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J429" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="430" spans="1:10" x14ac:dyDescent="0.2">
@@ -12573,7 +13230,7 @@
         <v>121</v>
       </c>
       <c r="C430" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D430" s="36" t="s">
         <v>655</v>
@@ -12587,8 +13244,11 @@
       <c r="H430" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I430" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J430" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="431" spans="1:10" x14ac:dyDescent="0.2">
@@ -12599,7 +13259,7 @@
         <v>121</v>
       </c>
       <c r="C431" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D431" s="36" t="s">
         <v>204</v>
@@ -12612,6 +13272,9 @@
       </c>
       <c r="H431" s="36" t="s">
         <v>656</v>
+      </c>
+      <c r="I431" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="432" spans="1:10" x14ac:dyDescent="0.2">
@@ -12622,7 +13285,7 @@
         <v>121</v>
       </c>
       <c r="C432" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D432" s="36" t="s">
         <v>655</v>
@@ -12636,8 +13299,11 @@
       <c r="H432" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I432" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J432" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="433" spans="1:10" x14ac:dyDescent="0.2">
@@ -12648,7 +13314,7 @@
         <v>121</v>
       </c>
       <c r="C433" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D433" s="36" t="s">
         <v>655</v>
@@ -12662,8 +13328,11 @@
       <c r="H433" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I433" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J433" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="434" spans="1:10" x14ac:dyDescent="0.2">
@@ -12674,7 +13343,7 @@
         <v>121</v>
       </c>
       <c r="C434" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D434" s="36" t="s">
         <v>654</v>
@@ -12688,11 +13357,11 @@
       <c r="H434" s="36" t="s">
         <v>657</v>
       </c>
-      <c r="I434" t="s">
-        <v>756</v>
+      <c r="I434" s="36" t="s">
+        <v>829</v>
       </c>
       <c r="J434" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="435" spans="1:10" x14ac:dyDescent="0.2">
@@ -12703,7 +13372,7 @@
         <v>121</v>
       </c>
       <c r="C435" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D435" s="36" t="s">
         <v>654</v>
@@ -12717,11 +13386,11 @@
       <c r="H435" s="36" t="s">
         <v>657</v>
       </c>
-      <c r="I435" t="s">
-        <v>756</v>
+      <c r="I435" s="36" t="s">
+        <v>829</v>
       </c>
       <c r="J435" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="436" spans="1:10" x14ac:dyDescent="0.2">
@@ -12732,7 +13401,7 @@
         <v>121</v>
       </c>
       <c r="C436" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D436" s="36" t="s">
         <v>654</v>
@@ -12746,11 +13415,11 @@
       <c r="H436" s="36" t="s">
         <v>657</v>
       </c>
-      <c r="I436" t="s">
-        <v>756</v>
+      <c r="I436" s="36" t="s">
+        <v>829</v>
       </c>
       <c r="J436" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="437" spans="1:10" x14ac:dyDescent="0.2">
@@ -12761,7 +13430,7 @@
         <v>121</v>
       </c>
       <c r="C437" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D437" s="36" t="s">
         <v>654</v>
@@ -12775,8 +13444,11 @@
       <c r="H437" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I437" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J437" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="438" spans="1:10" x14ac:dyDescent="0.2">
@@ -12787,7 +13459,7 @@
         <v>121</v>
       </c>
       <c r="C438" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D438" s="36" t="s">
         <v>654</v>
@@ -12801,8 +13473,11 @@
       <c r="H438" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I438" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J438" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="439" spans="1:10" x14ac:dyDescent="0.2">
@@ -12813,7 +13488,7 @@
         <v>121</v>
       </c>
       <c r="C439" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D439" s="36" t="s">
         <v>654</v>
@@ -12827,8 +13502,11 @@
       <c r="H439" s="36" t="s">
         <v>658</v>
       </c>
+      <c r="I439" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J439" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="440" spans="1:10" x14ac:dyDescent="0.2">
@@ -12839,7 +13517,7 @@
         <v>121</v>
       </c>
       <c r="C440" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D440" s="36" t="s">
         <v>654</v>
@@ -12853,8 +13531,11 @@
       <c r="H440" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I440" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J440" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="441" spans="1:10" x14ac:dyDescent="0.2">
@@ -12865,7 +13546,7 @@
         <v>121</v>
       </c>
       <c r="C441" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D441" s="36" t="s">
         <v>654</v>
@@ -12879,8 +13560,11 @@
       <c r="H441" s="36" t="s">
         <v>656</v>
       </c>
+      <c r="I441" s="36" t="s">
+        <v>829</v>
+      </c>
       <c r="J441" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="442" spans="1:10" x14ac:dyDescent="0.2">
@@ -12891,7 +13575,7 @@
         <v>121</v>
       </c>
       <c r="C442" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D442" s="36" t="s">
         <v>204</v>
@@ -12904,6 +13588,9 @@
       </c>
       <c r="H442" s="36" t="s">
         <v>656</v>
+      </c>
+      <c r="I442" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="443" spans="1:10" x14ac:dyDescent="0.2">
@@ -12914,7 +13601,7 @@
         <v>121</v>
       </c>
       <c r="C443" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D443" s="36" t="s">
         <v>204</v>
@@ -12927,6 +13614,9 @@
       </c>
       <c r="H443" s="36" t="s">
         <v>656</v>
+      </c>
+      <c r="I443" s="36" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="444" spans="1:10" x14ac:dyDescent="0.2">
@@ -13029,10 +13719,13 @@
         <v>300</v>
       </c>
       <c r="H448" s="36" t="s">
-        <v>759</v>
+        <v>758</v>
+      </c>
+      <c r="I448" s="36" t="s">
+        <v>826</v>
       </c>
       <c r="J448" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="449" spans="1:10" x14ac:dyDescent="0.2">
@@ -13055,10 +13748,13 @@
         <v>300</v>
       </c>
       <c r="H449" s="36" t="s">
-        <v>759</v>
+        <v>758</v>
+      </c>
+      <c r="I449" s="36" t="s">
+        <v>826</v>
       </c>
       <c r="J449" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="450" spans="1:10" x14ac:dyDescent="0.2">
@@ -13081,10 +13777,13 @@
         <v>300</v>
       </c>
       <c r="H450" s="36" t="s">
-        <v>759</v>
+        <v>758</v>
+      </c>
+      <c r="I450" s="36" t="s">
+        <v>826</v>
       </c>
       <c r="J450" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="451" spans="1:10" x14ac:dyDescent="0.2">
@@ -13107,10 +13806,13 @@
         <v>300</v>
       </c>
       <c r="H451" s="36" t="s">
-        <v>759</v>
+        <v>758</v>
+      </c>
+      <c r="I451" s="36" t="s">
+        <v>826</v>
       </c>
       <c r="J451" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="452" spans="1:10" x14ac:dyDescent="0.2">
@@ -13133,10 +13835,13 @@
         <v>300</v>
       </c>
       <c r="H452" s="36" t="s">
-        <v>759</v>
+        <v>758</v>
+      </c>
+      <c r="I452" s="36" t="s">
+        <v>826</v>
       </c>
       <c r="J452" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="453" spans="1:10" x14ac:dyDescent="0.2">
@@ -13159,10 +13864,13 @@
         <v>300</v>
       </c>
       <c r="H453" s="36" t="s">
+        <v>758</v>
+      </c>
+      <c r="I453" s="36" t="s">
+        <v>826</v>
+      </c>
+      <c r="J453" t="s">
         <v>759</v>
-      </c>
-      <c r="J453" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="454" spans="1:10" x14ac:dyDescent="0.2">
@@ -13185,10 +13893,13 @@
         <v>300</v>
       </c>
       <c r="H454" s="36" t="s">
+        <v>758</v>
+      </c>
+      <c r="I454" s="36" t="s">
+        <v>826</v>
+      </c>
+      <c r="J454" t="s">
         <v>759</v>
-      </c>
-      <c r="J454" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="455" spans="1:10" x14ac:dyDescent="0.2">
@@ -13211,10 +13922,13 @@
         <v>300</v>
       </c>
       <c r="H455" s="36" t="s">
+        <v>758</v>
+      </c>
+      <c r="I455" s="36" t="s">
+        <v>826</v>
+      </c>
+      <c r="J455" t="s">
         <v>759</v>
-      </c>
-      <c r="J455" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="456" spans="1:10" x14ac:dyDescent="0.2">
@@ -13237,10 +13951,13 @@
         <v>300</v>
       </c>
       <c r="H456" s="36" t="s">
+        <v>758</v>
+      </c>
+      <c r="I456" s="36" t="s">
+        <v>826</v>
+      </c>
+      <c r="J456" t="s">
         <v>759</v>
-      </c>
-      <c r="J456" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="457" spans="1:10" x14ac:dyDescent="0.2">
@@ -13263,10 +13980,13 @@
         <v>300</v>
       </c>
       <c r="H457" s="36" t="s">
+        <v>758</v>
+      </c>
+      <c r="I457" s="36" t="s">
+        <v>826</v>
+      </c>
+      <c r="J457" t="s">
         <v>759</v>
-      </c>
-      <c r="J457" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="458" spans="1:10" x14ac:dyDescent="0.2">
@@ -13289,7 +14009,10 @@
         <v>150</v>
       </c>
       <c r="H458" s="36" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I458" s="36" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="459" spans="1:10" x14ac:dyDescent="0.2">
@@ -13312,7 +14035,10 @@
         <v>150</v>
       </c>
       <c r="H459" s="36" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I459" s="36" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="460" spans="1:10" x14ac:dyDescent="0.2">
@@ -13335,7 +14061,10 @@
         <v>150</v>
       </c>
       <c r="H460" s="36" t="s">
-        <v>758</v>
+        <v>757</v>
+      </c>
+      <c r="I460" s="36" t="s">
+        <v>826</v>
       </c>
     </row>
     <row r="461" spans="1:10" x14ac:dyDescent="0.2">
@@ -13418,7 +14147,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="465" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="465" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A465" s="45" t="s">
         <v>683</v>
       </c>
@@ -13438,7 +14167,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="466" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="466" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A466" s="45" t="s">
         <v>684</v>
       </c>
@@ -13458,7 +14187,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="467" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="467" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A467" s="36" t="s">
         <v>685</v>
       </c>
@@ -13477,8 +14206,11 @@
       <c r="F467" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="468" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I467" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="468" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A468" s="36" t="s">
         <v>686</v>
       </c>
@@ -13497,8 +14229,11 @@
       <c r="F468" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="469" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I468" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="469" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A469" s="36" t="s">
         <v>687</v>
       </c>
@@ -13517,8 +14252,11 @@
       <c r="F469" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="470" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I469" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="470" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A470" s="36" t="s">
         <v>688</v>
       </c>
@@ -13537,8 +14275,11 @@
       <c r="F470" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="471" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I470" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="471" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A471" s="36" t="s">
         <v>689</v>
       </c>
@@ -13557,8 +14298,11 @@
       <c r="F471" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="472" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I471" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="472" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A472" s="36" t="s">
         <v>690</v>
       </c>
@@ -13577,8 +14321,11 @@
       <c r="F472" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="473" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I472" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="473" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A473" s="36" t="s">
         <v>691</v>
       </c>
@@ -13597,8 +14344,11 @@
       <c r="F473" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="474" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I473" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="474" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A474" s="36" t="s">
         <v>692</v>
       </c>
@@ -13617,8 +14367,11 @@
       <c r="F474" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="475" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I474" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="475" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A475" s="36" t="s">
         <v>693</v>
       </c>
@@ -13637,8 +14390,11 @@
       <c r="F475" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="476" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I475" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="476" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A476" s="36" t="s">
         <v>694</v>
       </c>
@@ -13657,8 +14413,11 @@
       <c r="F476" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="477" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I476" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="477" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A477" s="36" t="s">
         <v>695</v>
       </c>
@@ -13677,8 +14436,11 @@
       <c r="F477" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="478" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I477" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="478" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A478" s="36" t="s">
         <v>696</v>
       </c>
@@ -13697,8 +14459,11 @@
       <c r="F478" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="479" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I478" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="479" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A479" s="36" t="s">
         <v>697</v>
       </c>
@@ -13717,8 +14482,11 @@
       <c r="F479" s="36">
         <v>300</v>
       </c>
-    </row>
-    <row r="480" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="I479" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="480" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A480" s="36" t="s">
         <v>698</v>
       </c>
@@ -13736,6 +14504,9 @@
       </c>
       <c r="F480" s="36">
         <v>300</v>
+      </c>
+      <c r="I480" t="s">
+        <v>831</v>
       </c>
     </row>
     <row r="481" spans="1:12" x14ac:dyDescent="0.2">
@@ -13757,6 +14528,9 @@
       <c r="F481" s="36">
         <v>300</v>
       </c>
+      <c r="I481" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="482" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A482" s="36" t="s">
@@ -13777,6 +14551,9 @@
       <c r="F482" s="36">
         <v>300</v>
       </c>
+      <c r="I482" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="483" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A483" s="36" t="s">
@@ -13797,6 +14574,9 @@
       <c r="F483" s="36">
         <v>300</v>
       </c>
+      <c r="I483" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="484" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A484" s="36" t="s">
@@ -13817,6 +14597,9 @@
       <c r="F484" s="36">
         <v>300</v>
       </c>
+      <c r="I484" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="485" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A485" s="36" t="s">
@@ -13837,6 +14620,9 @@
       <c r="F485" s="36">
         <v>300</v>
       </c>
+      <c r="I485" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="486" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A486" s="36" t="s">
@@ -13857,6 +14643,9 @@
       <c r="F486" s="36">
         <v>300</v>
       </c>
+      <c r="I486" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="487" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A487" s="36" t="s">
@@ -13877,6 +14666,9 @@
       <c r="F487" s="36">
         <v>300</v>
       </c>
+      <c r="I487" t="s">
+        <v>831</v>
+      </c>
     </row>
     <row r="488" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A488" s="49" t="s">
@@ -13897,6 +14689,9 @@
       <c r="F488" s="36">
         <v>100</v>
       </c>
+      <c r="I488" t="s">
+        <v>833</v>
+      </c>
       <c r="L488" t="s">
         <v>748</v>
       </c>
@@ -13920,6 +14715,9 @@
       <c r="F489" s="36">
         <v>100</v>
       </c>
+      <c r="I489" t="s">
+        <v>833</v>
+      </c>
       <c r="L489" t="s">
         <v>748</v>
       </c>
@@ -13943,6 +14741,9 @@
       <c r="F490" s="36">
         <v>100</v>
       </c>
+      <c r="I490" t="s">
+        <v>833</v>
+      </c>
       <c r="L490" t="s">
         <v>748</v>
       </c>
@@ -13966,6 +14767,9 @@
       <c r="F491" s="36">
         <v>100</v>
       </c>
+      <c r="I491" t="s">
+        <v>833</v>
+      </c>
       <c r="L491" t="s">
         <v>748</v>
       </c>
@@ -13989,6 +14793,9 @@
       <c r="F492" s="36">
         <v>100</v>
       </c>
+      <c r="I492" t="s">
+        <v>833</v>
+      </c>
       <c r="L492" t="s">
         <v>748</v>
       </c>
@@ -14012,6 +14819,9 @@
       <c r="F493" s="36">
         <v>100</v>
       </c>
+      <c r="I493" t="s">
+        <v>833</v>
+      </c>
       <c r="L493" t="s">
         <v>748</v>
       </c>
@@ -14035,6 +14845,9 @@
       <c r="F494" s="36">
         <v>100</v>
       </c>
+      <c r="I494" t="s">
+        <v>833</v>
+      </c>
       <c r="L494" t="s">
         <v>748</v>
       </c>
@@ -14058,6 +14871,9 @@
       <c r="F495" s="36">
         <v>100</v>
       </c>
+      <c r="I495" t="s">
+        <v>833</v>
+      </c>
       <c r="L495" t="s">
         <v>748</v>
       </c>
@@ -14081,6 +14897,9 @@
       <c r="F496" s="36">
         <v>100</v>
       </c>
+      <c r="I496" t="s">
+        <v>833</v>
+      </c>
       <c r="L496" t="s">
         <v>748</v>
       </c>
@@ -14107,6 +14926,9 @@
       <c r="H497" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I497" t="s">
+        <v>833</v>
+      </c>
       <c r="L497" t="s">
         <v>748</v>
       </c>
@@ -14133,6 +14955,9 @@
       <c r="H498" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I498" t="s">
+        <v>833</v>
+      </c>
       <c r="L498" t="s">
         <v>748</v>
       </c>
@@ -14159,6 +14984,9 @@
       <c r="H499" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I499" t="s">
+        <v>833</v>
+      </c>
       <c r="L499" t="s">
         <v>748</v>
       </c>
@@ -14185,6 +15013,9 @@
       <c r="H500" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I500" t="s">
+        <v>833</v>
+      </c>
       <c r="L500" t="s">
         <v>748</v>
       </c>
@@ -14211,6 +15042,9 @@
       <c r="H501" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I501" t="s">
+        <v>833</v>
+      </c>
       <c r="L501" t="s">
         <v>748</v>
       </c>
@@ -14237,6 +15071,9 @@
       <c r="H502" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I502" t="s">
+        <v>833</v>
+      </c>
       <c r="L502" t="s">
         <v>748</v>
       </c>
@@ -14260,6 +15097,9 @@
       <c r="F503" s="36">
         <v>100</v>
       </c>
+      <c r="I503" t="s">
+        <v>833</v>
+      </c>
       <c r="L503" t="s">
         <v>748</v>
       </c>
@@ -14286,6 +15126,9 @@
       <c r="H504" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I504" t="s">
+        <v>833</v>
+      </c>
       <c r="L504" t="s">
         <v>748</v>
       </c>
@@ -14312,6 +15155,9 @@
       <c r="H505" s="36" t="s">
         <v>752</v>
       </c>
+      <c r="I505" t="s">
+        <v>833</v>
+      </c>
       <c r="L505" t="s">
         <v>748</v>
       </c>
@@ -14335,6 +15181,9 @@
       <c r="F506" s="36">
         <v>202</v>
       </c>
+      <c r="I506" t="s">
+        <v>834</v>
+      </c>
     </row>
     <row r="507" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A507" s="36" t="s">
@@ -14355,6 +15204,9 @@
       <c r="F507" s="36">
         <v>202</v>
       </c>
+      <c r="I507" t="s">
+        <v>834</v>
+      </c>
     </row>
     <row r="508" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A508" s="36" t="s">
@@ -14375,6 +15227,9 @@
       <c r="F508" s="36">
         <v>202</v>
       </c>
+      <c r="I508" t="s">
+        <v>834</v>
+      </c>
     </row>
     <row r="509" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A509" s="36" t="s">
@@ -14395,6 +15250,9 @@
       <c r="F509" s="36">
         <v>202</v>
       </c>
+      <c r="I509" t="s">
+        <v>834</v>
+      </c>
     </row>
     <row r="510" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A510" s="36" t="s">
@@ -14415,6 +15273,9 @@
       <c r="F510" s="36">
         <v>202</v>
       </c>
+      <c r="I510" t="s">
+        <v>834</v>
+      </c>
     </row>
     <row r="511" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A511" s="36" t="s">
@@ -14434,6 +15295,9 @@
       </c>
       <c r="F511" s="36">
         <v>202</v>
+      </c>
+      <c r="I511" t="s">
+        <v>834</v>
       </c>
     </row>
     <row r="515" spans="2:8" x14ac:dyDescent="0.2">
@@ -14828,7 +15692,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FF710BC-207F-AF4F-A439-3F607FA565E9}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -14842,7 +15706,7 @@
     <col min="13" max="13" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -14864,8 +15728,11 @@
       <c r="H1" s="1" t="s">
         <v>730</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="I1" s="1" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="s">
         <v>53</v>
       </c>
@@ -14888,8 +15755,11 @@
       <c r="H2" s="25" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="I2" s="25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>109</v>
       </c>
@@ -14911,8 +15781,11 @@
       <c r="H3" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="68" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I3" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="68" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="42" t="s">
         <v>55</v>
       </c>
@@ -14938,7 +15811,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
         <v>55</v>
       </c>
@@ -14961,8 +15834,11 @@
       <c r="H5" s="25" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="I5" s="25" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
         <v>55</v>
       </c>
@@ -14987,8 +15863,11 @@
       <c r="H6" s="25" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="I6" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>68</v>
       </c>
@@ -15007,11 +15886,17 @@
       <c r="F7" t="s">
         <v>178</v>
       </c>
+      <c r="G7" t="s">
+        <v>827</v>
+      </c>
       <c r="H7" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="I7" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>68</v>
       </c>
@@ -15030,11 +15915,17 @@
       <c r="F8" t="s">
         <v>178</v>
       </c>
+      <c r="G8" t="s">
+        <v>825</v>
+      </c>
       <c r="H8" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="I8" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="32" t="s">
         <v>121</v>
       </c>
@@ -15059,8 +15950,11 @@
       <c r="H9" s="25" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I9" s="25" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="37" t="s">
         <v>121</v>
       </c>
@@ -15086,7 +15980,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" s="32" t="s">
         <v>121</v>
       </c>
@@ -15109,8 +16003,11 @@
       <c r="H11" s="25" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="51" hidden="1" x14ac:dyDescent="0.2">
+      <c r="I11" s="25" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="37" t="s">
         <v>125</v>
       </c>
@@ -15134,7 +16031,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>125</v>
       </c>
@@ -15159,8 +16056,11 @@
       <c r="H13" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="I13" s="25" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
         <v>731</v>
       </c>
@@ -15176,7 +16076,7 @@
       <c r="E14" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="33" t="s">
         <v>147</v>
       </c>
       <c r="G14" s="25" t="s">
@@ -15185,8 +16085,11 @@
       <c r="H14" s="25" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="I14" s="25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>202</v>
       </c>
@@ -15208,8 +16111,11 @@
       <c r="H15" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="I15" s="25" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>149</v>
       </c>
@@ -15230,6 +16136,9 @@
       </c>
       <c r="H16" t="s">
         <v>205</v>
+      </c>
+      <c r="I16" s="25" t="s">
+        <v>827</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -15253,13 +16162,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B21" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
   </sheetData>
@@ -15314,6 +16223,7 @@
     <hyperlink ref="B15" r:id="rId31" location="s1" xr:uid="{9BE0D8A7-9265-8642-873F-D3EFCA103F88}"/>
     <hyperlink ref="D15" r:id="rId32" xr:uid="{10FAA8A4-AA39-A945-831D-13348C3E39A4}"/>
     <hyperlink ref="D21" r:id="rId33" xr:uid="{FE9DC421-D5CE-8646-B5EF-C31D94D32565}"/>
+    <hyperlink ref="F14" r:id="rId34" location="s2" xr:uid="{BD48CE36-B249-9645-985C-74D9B28B1413}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -15330,209 +16240,209 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>782</v>
+      </c>
+      <c r="B1" t="s">
         <v>783</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>784</v>
-      </c>
-      <c r="C1" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>785</v>
+      </c>
+      <c r="B2" t="s">
         <v>786</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>787</v>
-      </c>
-      <c r="C2" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>788</v>
+      </c>
+      <c r="B3" t="s">
         <v>789</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>790</v>
-      </c>
-      <c r="C3" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>791</v>
+      </c>
+      <c r="B4" t="s">
+        <v>789</v>
+      </c>
+      <c r="C4" t="s">
         <v>792</v>
-      </c>
-      <c r="B4" t="s">
-        <v>790</v>
-      </c>
-      <c r="C4" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>793</v>
+      </c>
+      <c r="B5" t="s">
         <v>794</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>795</v>
-      </c>
-      <c r="C5" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>796</v>
+      </c>
+      <c r="B6" t="s">
         <v>797</v>
-      </c>
-      <c r="B6" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B7" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>799</v>
+      </c>
+      <c r="B8" t="s">
+        <v>797</v>
+      </c>
+      <c r="C8" t="s">
         <v>800</v>
-      </c>
-      <c r="B8" t="s">
-        <v>798</v>
-      </c>
-      <c r="C8" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>801</v>
+      </c>
+      <c r="B9" t="s">
+        <v>786</v>
+      </c>
+      <c r="C9" t="s">
         <v>802</v>
-      </c>
-      <c r="B9" t="s">
-        <v>787</v>
-      </c>
-      <c r="C9" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>803</v>
+      </c>
+      <c r="B10" t="s">
+        <v>789</v>
+      </c>
+      <c r="C10" t="s">
         <v>804</v>
-      </c>
-      <c r="B10" t="s">
-        <v>790</v>
-      </c>
-      <c r="C10" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>805</v>
+      </c>
+      <c r="B11" t="s">
+        <v>794</v>
+      </c>
+      <c r="C11" t="s">
         <v>806</v>
-      </c>
-      <c r="B11" t="s">
-        <v>795</v>
-      </c>
-      <c r="C11" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>807</v>
+      </c>
+      <c r="B12" t="s">
+        <v>797</v>
+      </c>
+      <c r="C12" t="s">
         <v>808</v>
-      </c>
-      <c r="B12" t="s">
-        <v>798</v>
-      </c>
-      <c r="C12" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>809</v>
+      </c>
+      <c r="B13" t="s">
+        <v>786</v>
+      </c>
+      <c r="C13" t="s">
         <v>810</v>
-      </c>
-      <c r="B13" t="s">
-        <v>787</v>
-      </c>
-      <c r="C13" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>811</v>
+      </c>
+      <c r="B14" t="s">
+        <v>789</v>
+      </c>
+      <c r="C14" t="s">
         <v>812</v>
-      </c>
-      <c r="B14" t="s">
-        <v>790</v>
-      </c>
-      <c r="C14" t="s">
-        <v>813</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>813</v>
+      </c>
+      <c r="B15" t="s">
+        <v>794</v>
+      </c>
+      <c r="C15" t="s">
         <v>814</v>
-      </c>
-      <c r="B15" t="s">
-        <v>795</v>
-      </c>
-      <c r="C15" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>815</v>
+      </c>
+      <c r="B16" t="s">
+        <v>786</v>
+      </c>
+      <c r="C16" t="s">
         <v>816</v>
-      </c>
-      <c r="B16" t="s">
-        <v>787</v>
-      </c>
-      <c r="C16" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>817</v>
+      </c>
+      <c r="B17" t="s">
+        <v>786</v>
+      </c>
+      <c r="C17" t="s">
         <v>818</v>
-      </c>
-      <c r="B17" t="s">
-        <v>787</v>
-      </c>
-      <c r="C17" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>819</v>
+      </c>
+      <c r="B18" t="s">
+        <v>794</v>
+      </c>
+      <c r="C18" t="s">
         <v>820</v>
-      </c>
-      <c r="B18" t="s">
-        <v>795</v>
-      </c>
-      <c r="C18" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="D32" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D33" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="34" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D34" s="19" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
   </sheetData>
@@ -15649,11 +16559,11 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="D7" t="s">
-        <v>764</v>
+      <c r="D7" s="19" t="s">
+        <v>763</v>
       </c>
       <c r="E7" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -15661,10 +16571,10 @@
         <v>739</v>
       </c>
       <c r="B8" t="s">
+        <v>764</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>765</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>766</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>738</v>
@@ -15679,6 +16589,7 @@
     <hyperlink ref="B6" r:id="rId5" location="sec0004" xr:uid="{C725378A-C201-5641-91B3-EC5CDEADF63B}"/>
     <hyperlink ref="D6" r:id="rId6" xr:uid="{4C1A6D6F-11AC-BF45-B9E8-BC73015E2AD9}"/>
     <hyperlink ref="D8" r:id="rId7" xr:uid="{127A4485-4D5D-1D42-B663-03B27FA7787F}"/>
+    <hyperlink ref="D7" r:id="rId8" xr:uid="{AFE3379E-5F1D-C949-8C20-81E119C2081F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>